<commit_message>
updated data and raw prompts
</commit_message>
<xml_diff>
--- a/legume X feature.xlsx
+++ b/legume X feature.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
   <si>
     <t xml:space="preserve">Yield per hectare</t>
   </si>
@@ -332,6 +332,24 @@
   </si>
   <si>
     <t xml:space="preserve">Crimson Clover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vicia lens (Lens culinaris)</t>
+  </si>
+  <si>
+    <t>Lentil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lathyrus sativus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indian Pea (Grass pea)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pisum sativum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pea (Garden pea)</t>
   </si>
 </sst>
 </file>
@@ -956,7 +974,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="24.00390625"/>
-    <col customWidth="1" min="2" max="2" width="16.421875"/>
+    <col customWidth="1" min="2" max="2" width="20.28125"/>
     <col customWidth="1" min="3" max="3" width="21.140625"/>
     <col customWidth="1" min="29" max="29" width="20.57421875"/>
   </cols>
@@ -1074,7 +1092,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" ht="180">
+    <row r="3" ht="135">
       <c r="C3" s="7" t="s">
         <v>37</v>
       </c>
@@ -1187,7 +1205,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" ht="30">
+    <row r="4" ht="15">
       <c r="A4" s="9" t="s">
         <v>74</v>
       </c>
@@ -1259,7 +1277,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="13" ht="60">
+    <row r="13" ht="30">
       <c r="A13" s="11" t="s">
         <v>92</v>
       </c>
@@ -1297,6 +1315,30 @@
       </c>
       <c r="B17" s="12" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18" t="s">
+        <v>102</v>
+      </c>
+      <c r="B18" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="A19" t="s">
+        <v>104</v>
+      </c>
+      <c r="B19" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>